<commit_message>
Add ai product improvement experiments
</commit_message>
<xml_diff>
--- a/ai-product-2/outputs/assignment2/assignment2_improvement_cycles.xlsx
+++ b/ai-product-2/outputs/assignment2/assignment2_improvement_cycles.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -681,6 +681,114 @@
         <v>0.5</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>metadata_filter_gemini_2_k8</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Infer company/year/filing type from the query, filter Gemini candidates, then generate with k=8</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.475</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.64</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>neighbor_context_gemini_2_k8</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Retrieve Gemini top-20, expand same-document page neighbors, then generate with k=8</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.38</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ontology_cluster_boost_gemini_2_k8</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Combine query metadata filters with same-document/page-neighbor cluster boosting, then generate with k=8</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.505</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.39</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>soft_metadata_boost_gemini_2_k8</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Retrieve Gemini top-30, softly boost query-matching metadata, then generate with k=8</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.5639999999999999</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.65</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>